<commit_message>
Explain Special Focus status and severity letters; mark Kingston closed
- Home list: a short key for Special Focus, Special Focus candidate, the abuse
  icon, harm citations, and the A-L severity groups; 'SFF candidate' badge now
  reads 'Special Focus candidate' with a hover explanation
- Facility pages: one-line explanation under a Special Focus badge
- About page: what Special Focus Facilities and candidates are, from CMS
  QSO-23-01-NH (revised January 2026)
- Builder: a facility details note starting 'Closed <Month> <Year>' marks a home
  closed even when CMS still lists it
- Kingston Center: closed January 2025 (PBN, Jan 28, 2025); owner group set to
  Centers Health Care, year sold cleared

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015nisUc5oGaBRT1cw14rGj4
</commit_message>
<xml_diff>
--- a/pipeline/facility_extras.xlsx
+++ b/pipeline/facility_extras.xlsx
@@ -3939,7 +3939,7 @@
       </c>
       <c r="C59" s="2" t="inlineStr">
         <is>
-          <t>AdviniaCare</t>
+          <t>Centers Health Care</t>
         </is>
       </c>
       <c r="D59" s="2" t="inlineStr">
@@ -3947,11 +3947,7 @@
           <t>corporate/investors</t>
         </is>
       </c>
-      <c r="E59" s="2" t="inlineStr">
-        <is>
-          <t>2026</t>
-        </is>
-      </c>
+      <c r="E59" s="2" t="n"/>
       <c r="F59" s="2" t="inlineStr"/>
       <c r="G59" s="2" t="inlineStr">
         <is>
@@ -3981,7 +3977,11 @@
           <t>ADVINIA</t>
         </is>
       </c>
-      <c r="S59" s="2" t="inlineStr"/>
+      <c r="S59" s="2" t="inlineStr">
+        <is>
+          <t>Closed January 2025, while it was being transferred to new owners. AdviniaCare never took it over.</t>
+        </is>
+      </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Build the hand-uploaded changes into the monthly update
The Oct 25 upload added PBJ Q1 2026 staffing, PBJ320 links, three
non-Medicare homes, and Scandinavian Home's closure directly to data.js.
The builder now produces all of them, so the monthly rebuild keeps them.
Scandinavian Home is marked "Closed 2025" from the facility extras notes.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015nisUc5oGaBRT1cw14rGj4
</commit_message>
<xml_diff>
--- a/pipeline/facility_extras.xlsx
+++ b/pipeline/facility_extras.xlsx
@@ -993,7 +993,11 @@
           <t>nonprofit</t>
         </is>
       </c>
-      <c r="S9" s="2" t="inlineStr"/>
+      <c r="S9" s="2" t="inlineStr">
+        <is>
+          <t>Closed 2025</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">

</xml_diff>